<commit_message>
Completing all the Accounts Managment User Stories- v1
</commit_message>
<xml_diff>
--- a/data/teachers.xlsx
+++ b/data/teachers.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahmed\OneDrive\Bureau\isamm-student-managment-platform\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44170D0B-EF37-4EE8-A216-F0BB09F37774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC7B53F0-7E30-4A01-9165-FEBBB4CCDFFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="810" yWindow="3900" windowWidth="24300" windowHeight="11460" xr2:uid="{AFD31129-8B99-4084-8265-242CB6D304A0}"/>
+    <workbookView xWindow="5625" yWindow="2745" windowWidth="19695" windowHeight="11505" xr2:uid="{AFD31129-8B99-4084-8265-242CB6D304A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="42">
   <si>
     <t>firstName</t>
   </si>
@@ -56,33 +56,15 @@
     <t>phone</t>
   </si>
   <si>
-    <t xml:space="preserve">password </t>
-  </si>
-  <si>
     <t>cv</t>
   </si>
   <si>
     <t>Ahmed</t>
   </si>
   <si>
-    <t>Ines</t>
-  </si>
-  <si>
-    <t>Masmoudi</t>
-  </si>
-  <si>
     <t>Gharbi</t>
   </si>
   <si>
-    <t>Amdouni</t>
-  </si>
-  <si>
-    <t>ahmed123</t>
-  </si>
-  <si>
-    <t>ines123</t>
-  </si>
-  <si>
     <t>ahmed_cv.pdf</t>
   </si>
   <si>
@@ -110,27 +92,6 @@
     <t>ilyes_cv.pdf</t>
   </si>
   <si>
-    <t>aziz_cv.pdf</t>
-  </si>
-  <si>
-    <t>ammar_cv.pdf</t>
-  </si>
-  <si>
-    <t>ines_cv.pdf</t>
-  </si>
-  <si>
-    <t>roua_cv.pdf</t>
-  </si>
-  <si>
-    <t>siwar_cv.pdf</t>
-  </si>
-  <si>
-    <t>nesrine_cv.pdf</t>
-  </si>
-  <si>
-    <t>emna_cv.pdf</t>
-  </si>
-  <si>
     <t>Amina</t>
   </si>
   <si>
@@ -155,30 +116,6 @@
     <t>Salah</t>
   </si>
   <si>
-    <t>Azouz</t>
-  </si>
-  <si>
-    <t>Abdlahmid</t>
-  </si>
-  <si>
-    <t>khalfalah</t>
-  </si>
-  <si>
-    <t>Rania</t>
-  </si>
-  <si>
-    <t>Samira</t>
-  </si>
-  <si>
-    <t>Nermine</t>
-  </si>
-  <si>
-    <t>Haj Gasem</t>
-  </si>
-  <si>
-    <t>Salwa</t>
-  </si>
-  <si>
     <t>Abdelwehed</t>
   </si>
   <si>
@@ -191,24 +128,12 @@
     <t>Hafsi</t>
   </si>
   <si>
-    <t>Lahmer</t>
-  </si>
-  <si>
-    <t>Bouchnak</t>
-  </si>
-  <si>
     <t>Jouini</t>
   </si>
   <si>
     <t>Mejri</t>
   </si>
   <si>
-    <t>Jendoubi</t>
-  </si>
-  <si>
-    <t>ahmedjendoubi@gmail.com</t>
-  </si>
-  <si>
     <t>salahmejri@gmail.com</t>
   </si>
   <si>
@@ -233,67 +158,10 @@
     <t>samirhafsi@gmail.com</t>
   </si>
   <si>
-    <t>azouzlahmer@gmail.com</t>
-  </si>
-  <si>
-    <t>abdlahmidbouchnak@gmail.com</t>
-  </si>
-  <si>
-    <t>ineskhalfalah@gmail.com</t>
-  </si>
-  <si>
-    <t>raniaamdouni@gmail.com</t>
-  </si>
-  <si>
-    <t>samiragharbi@gmail.com</t>
-  </si>
-  <si>
-    <t>salwamasmoudi@gmail.com</t>
-  </si>
-  <si>
-    <t>salah123</t>
-  </si>
-  <si>
-    <t>mondher113</t>
-  </si>
-  <si>
-    <t>dali113</t>
-  </si>
-  <si>
-    <t>amina123</t>
-  </si>
-  <si>
-    <t>hafedh123</t>
-  </si>
-  <si>
-    <t>sonia133</t>
-  </si>
-  <si>
-    <t>fatma133</t>
-  </si>
-  <si>
-    <t>samir133</t>
-  </si>
-  <si>
-    <t>azouz123</t>
-  </si>
-  <si>
-    <t>abdlahmid123</t>
-  </si>
-  <si>
-    <t>rania113</t>
-  </si>
-  <si>
-    <t>samira113</t>
-  </si>
-  <si>
-    <t>nermine113</t>
-  </si>
-  <si>
-    <t>salwa113</t>
-  </si>
-  <si>
-    <t>nerminehajgasem@gmail.com</t>
+    <t>aahmedgafsi@gmail.com</t>
+  </si>
+  <si>
+    <t>gafsi</t>
   </si>
 </sst>
 </file>
@@ -345,12 +213,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
@@ -720,14 +587,11 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
       </c>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -737,417 +601,236 @@
       <c r="A2">
         <v>22222222</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2">
         <v>36902</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2">
+        <v>41</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F2">
         <v>25234567</v>
       </c>
-      <c r="H2" t="s">
-        <v>15</v>
+      <c r="G2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>22222223</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>36903</v>
       </c>
       <c r="C3" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="D3" t="s">
-        <v>54</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="F3" t="s">
-        <v>71</v>
-      </c>
-      <c r="G3">
+        <v>31</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3">
         <v>25234568</v>
       </c>
-      <c r="H3" t="s">
-        <v>16</v>
+      <c r="G3" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>22222224</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>36904</v>
       </c>
       <c r="C4" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>53</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="F4" t="s">
-        <v>72</v>
-      </c>
-      <c r="G4">
+        <v>30</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4">
         <v>25234579</v>
       </c>
-      <c r="H4" t="s">
-        <v>17</v>
+      <c r="G4" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>22222225</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>36905</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="F5" t="s">
-        <v>73</v>
-      </c>
-      <c r="G5">
+        <v>26</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5">
         <v>25234581</v>
       </c>
-      <c r="H5" t="s">
-        <v>18</v>
+      <c r="G5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>22222226</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <v>36906</v>
       </c>
       <c r="C6" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="D6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="F6" t="s">
-        <v>74</v>
-      </c>
-      <c r="G6">
+        <v>26</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6">
         <v>25234582</v>
       </c>
-      <c r="H6" t="s">
-        <v>19</v>
+      <c r="G6" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>22222227</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="2">
         <v>36907</v>
       </c>
       <c r="C7" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="D7" t="s">
-        <v>48</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="F7" t="s">
-        <v>75</v>
-      </c>
-      <c r="G7">
+        <v>27</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7">
         <v>25234583</v>
       </c>
-      <c r="H7" t="s">
-        <v>20</v>
+      <c r="G7" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>22222228</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="2">
         <v>36908</v>
       </c>
       <c r="C8" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="D8" t="s">
-        <v>49</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="F8" t="s">
-        <v>76</v>
-      </c>
-      <c r="G8">
+        <v>28</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8">
         <v>25234584</v>
       </c>
-      <c r="H8" t="s">
-        <v>21</v>
+      <c r="G8" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>22222229</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="2">
         <v>36909</v>
       </c>
       <c r="C9" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="D9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="F9" t="s">
-        <v>77</v>
-      </c>
-      <c r="G9">
+        <v>8</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9">
         <v>25234585</v>
       </c>
-      <c r="H9" t="s">
-        <v>22</v>
+      <c r="G9" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>22222230</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="2">
         <v>36910</v>
       </c>
       <c r="C10" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="D10" t="s">
-        <v>50</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="F10" t="s">
-        <v>78</v>
-      </c>
-      <c r="G10">
+        <v>29</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F10">
         <v>25234586</v>
       </c>
-      <c r="H10" t="s">
-        <v>23</v>
+      <c r="G10" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>22222231</v>
-      </c>
-      <c r="B11" s="3">
-        <v>36911</v>
-      </c>
-      <c r="C11" t="s">
-        <v>39</v>
-      </c>
-      <c r="D11" t="s">
-        <v>51</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="F11" t="s">
-        <v>79</v>
-      </c>
-      <c r="G11">
-        <v>25234587</v>
-      </c>
-      <c r="H11" t="s">
-        <v>24</v>
-      </c>
+      <c r="B11" s="2"/>
+      <c r="E11" s="3"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>22222232</v>
-      </c>
-      <c r="B12" s="3">
-        <v>36912</v>
-      </c>
-      <c r="C12" t="s">
-        <v>40</v>
-      </c>
-      <c r="D12" t="s">
-        <v>52</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="F12" t="s">
-        <v>80</v>
-      </c>
-      <c r="G12">
-        <v>25234588</v>
-      </c>
-      <c r="H12" t="s">
-        <v>25</v>
-      </c>
+      <c r="B12" s="2"/>
+      <c r="E12" s="3"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>22222233</v>
-      </c>
-      <c r="B13" s="3">
-        <v>36913</v>
-      </c>
-      <c r="C13" t="s">
-        <v>9</v>
-      </c>
-      <c r="D13" t="s">
-        <v>41</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="F13" t="s">
-        <v>14</v>
-      </c>
-      <c r="G13">
-        <v>25234589</v>
-      </c>
-      <c r="H13" t="s">
-        <v>26</v>
-      </c>
+      <c r="B13" s="2"/>
+      <c r="E13" s="3"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>22222234</v>
-      </c>
-      <c r="B14" s="3">
-        <v>36914</v>
-      </c>
-      <c r="C14" t="s">
-        <v>42</v>
-      </c>
-      <c r="D14" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="F14" t="s">
-        <v>81</v>
-      </c>
-      <c r="G14">
-        <v>25234589</v>
-      </c>
-      <c r="H14" t="s">
-        <v>27</v>
-      </c>
+      <c r="B14" s="2"/>
+      <c r="E14" s="3"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>22222235</v>
-      </c>
-      <c r="B15" s="3">
-        <v>36915</v>
-      </c>
-      <c r="C15" t="s">
-        <v>43</v>
-      </c>
-      <c r="D15" t="s">
-        <v>11</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="F15" t="s">
-        <v>82</v>
-      </c>
-      <c r="G15">
-        <v>25234589</v>
-      </c>
-      <c r="H15" t="s">
-        <v>28</v>
-      </c>
+      <c r="B15" s="2"/>
+      <c r="E15" s="3"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>22222236</v>
-      </c>
-      <c r="B16" s="3">
-        <v>36916</v>
-      </c>
-      <c r="C16" t="s">
-        <v>44</v>
-      </c>
-      <c r="D16" t="s">
-        <v>45</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="F16" t="s">
-        <v>83</v>
-      </c>
-      <c r="G16">
-        <v>25234589</v>
-      </c>
-      <c r="H16" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>22222237</v>
-      </c>
-      <c r="B17" s="3">
-        <v>36917</v>
-      </c>
-      <c r="C17" t="s">
-        <v>46</v>
-      </c>
-      <c r="D17" t="s">
-        <v>10</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="F17" t="s">
-        <v>84</v>
-      </c>
-      <c r="G17">
-        <v>25234589</v>
-      </c>
-      <c r="H17" t="s">
-        <v>30</v>
-      </c>
+      <c r="B16" s="2"/>
+      <c r="E16" s="3"/>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B17" s="2"/>
+      <c r="E17" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1160,15 +843,8 @@
     <hyperlink ref="E8" r:id="rId7" xr:uid="{45A11D35-1DD1-47EB-885A-3FBBC8E383DF}"/>
     <hyperlink ref="E9" r:id="rId8" xr:uid="{9BE2A3C0-CAEB-4FC2-A324-223A09580BB5}"/>
     <hyperlink ref="E10" r:id="rId9" xr:uid="{CB0534FE-8161-4A92-A92B-0F8B57436513}"/>
-    <hyperlink ref="E11" r:id="rId10" xr:uid="{D10F77CC-5265-4966-B60C-DF3C54D39C66}"/>
-    <hyperlink ref="E12" r:id="rId11" xr:uid="{EC096393-2B18-4726-A951-3761F61F56E7}"/>
-    <hyperlink ref="E13" r:id="rId12" xr:uid="{16695906-B4CF-4AE6-8FBB-32F29B505AAD}"/>
-    <hyperlink ref="E14" r:id="rId13" xr:uid="{DED1F55E-22B1-4EDD-86DF-9A5470795B65}"/>
-    <hyperlink ref="E15" r:id="rId14" xr:uid="{0B34521D-BC9B-4E26-9EEA-4C6743AEC8A8}"/>
-    <hyperlink ref="E17" r:id="rId15" xr:uid="{B435A633-CE3F-469B-887D-0B267F119DE2}"/>
-    <hyperlink ref="E16" r:id="rId16" xr:uid="{57FAC454-C506-48A2-BD26-8E2E3C2DBBFC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId17"/>
+  <pageSetup orientation="portrait" r:id="rId10"/>
 </worksheet>
 </file>
</xml_diff>